<commit_message>
Pushing the changes for bap
</commit_message>
<xml_diff>
--- a/src/main/resources/static/EventAttendedRepository.xlsx
+++ b/src/main/resources/static/EventAttendedRepository.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tanishq\Events\tanishq_events\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sudhi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DC6B4DE3-9EC3-42ED-91B8-5C3C512BF91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1FE03D2-B574-4979-8E9B-39B4505407C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{27BD6C3F-0E7E-4759-BD34-D89B86A738F6}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Name</t>
   </si>
@@ -33,24 +33,44 @@
     <t>Phone</t>
   </si>
   <si>
-    <t>customer name</t>
-  </si>
-  <si>
-    <t>customer mobile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">like Diamond or Gold </t>
-  </si>
-  <si>
-    <t>Customer choise (Diamond/Gold/Both)</t>
+    <t>first time for event</t>
+  </si>
+  <si>
+    <t>RSO Name</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>Alok</t>
+  </si>
+  <si>
+    <t>Sudhir</t>
+  </si>
+  <si>
+    <t>Ramesh</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Mohan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -78,8 +98,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -394,37 +418,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B79FB2C8-1B72-4E21-931E-AA9AA71A0F58}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.88671875" customWidth="1"/>
     <col min="2" max="2" width="35.77734375" customWidth="1"/>
     <col min="3" max="3" width="27.44140625" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>1234567890</v>
+      </c>
+      <c r="C2" t="s">
         <v>4</v>
       </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>1234567890</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="G1:XFD1048576"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>